<commit_message>
feat: Implement official approved weights (10% Hozori, 30% Majazi [40% training pool], 50% Khalagh [capped at 100%], 10% Tolidat)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/نمرات_عملکرد_2ماهه.xlsx
+++ b/نمرات_عملکرد_2ماهه.xlsx
@@ -10,7 +10,7 @@
     <sheet name="فقط نام و نمره (ساده)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="جدول نمرات و تحلیل ماه‌ها" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="رتبه‌بندی استانی" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="مستندات شاخص‌ها" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ریز مستندات و اوزان شاخص‌ها" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -64,7 +64,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -87,18 +87,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
         <bgColor rgb="00FEE2E2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
-        <bgColor rgb="00D1FAE5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -134,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -160,13 +148,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -580,7 +562,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5">
@@ -780,7 +762,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>86</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25">
@@ -820,7 +802,7 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>85.2</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29">
@@ -893,13 +875,13 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>جدول ارزیابی عملکرد ۲ ماهه نواحی نسرا (مقیاس ۷۰ تا ۱۰۰ | ۳ سطح کیفی)</t>
+          <t>جدول ارزیابی عملکرد ۲ ماهه نواحی نسرا (۱۰٪ حضوری، ۳۰٪ مجازی، ۵۰٪ خلاقانه، ۱۰٪ تولیدات)</t>
         </is>
       </c>
     </row>
@@ -1016,24 +998,26 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>عالی</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>1</v>
+        <v>70</v>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>2 از 2 ماه</t>
+          <t>0 از 2 ماه</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>کامل (2 از 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
         </is>
       </c>
     </row>
@@ -1674,24 +1658,26 @@
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>86</v>
-      </c>
-      <c r="D26" s="10" t="inlineStr">
-        <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>2</v>
+        <v>70</v>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>1 از 2 ماه</t>
+          <t>0 از 2 ماه</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>کسری: 1 از 2 ماه (عدم فعالیت در: مرداد 1405)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
         </is>
       </c>
     </row>
@@ -1804,24 +1790,26 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>85.2</v>
-      </c>
-      <c r="D30" s="10" t="inlineStr">
-        <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="n">
-        <v>3</v>
+        <v>70</v>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>1 از 2 ماه</t>
+          <t>0 از 2 ماه</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>کسری: 1 از 2 ماه (عدم فعالیت در: شهریور 1405)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
         </is>
       </c>
     </row>
@@ -2023,118 +2011,124 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>رتبه</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>نام ناحیه (شهرستان)</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>نمره عملکرد (۷۰-۱۰۰)</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>سطح کیفی</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
-        <is>
-          <t>درصد تحقق اهداف</t>
-        </is>
-      </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>درصد تحقق وزنی</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>تعداد ماه‌های ارسالی</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>1</v>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>آران و بیدگل</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>0 از 2 ماه</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>امام حسین(ع)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>0 از 2 ماه</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
           <t>امام رضا(ع)</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>عالی</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>103.2%</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>2 از 2 ماه</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>کاشان</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>86</v>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>53.4%</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>1 از 2 ماه</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>مبارکه</t>
-        </is>
-      </c>
       <c r="C6" s="6" t="n">
-        <v>85.2</v>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+        <v>70</v>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>50.7%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>1 از 2 ماه</t>
+          <t>0 از 2 ماه</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2140,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>آران و بیدگل</t>
+          <t>امام صادق(ع)</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
@@ -2176,7 +2170,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>امام حسین(ع)</t>
+          <t>امام علی(ع)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
@@ -2206,7 +2200,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>امام صادق(ع)</t>
+          <t>اردستان</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
@@ -2236,7 +2230,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>امام علی(ع)</t>
+          <t>برخوار</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
@@ -2266,7 +2260,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>اردستان</t>
+          <t>بویین و میاندشت</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
@@ -2296,7 +2290,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>برخوار</t>
+          <t>تیران و کرون</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
@@ -2326,7 +2320,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>بویین و میاندشت</t>
+          <t>جرقویه</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
@@ -2356,7 +2350,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>تیران و کرون</t>
+          <t>چادگان</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
@@ -2386,7 +2380,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>جرقویه</t>
+          <t>خمینی شهر</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
@@ -2416,7 +2410,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>چادگان</t>
+          <t>خوانسار</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
@@ -2446,7 +2440,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>خمینی شهر</t>
+          <t>خور و بیابانک</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
@@ -2476,7 +2470,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>خوانسار</t>
+          <t>درچه</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
@@ -2506,7 +2500,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>خور و بیابانک</t>
+          <t>دهاقان</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
@@ -2536,7 +2530,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>درچه</t>
+          <t>سمیرم</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
@@ -2566,7 +2560,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>دهاقان</t>
+          <t>شاهین شهر</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
@@ -2596,7 +2590,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>سمیرم</t>
+          <t>شهرضا</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
@@ -2626,7 +2620,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>شاهین شهر</t>
+          <t>فریدن</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
@@ -2656,7 +2650,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>شهرضا</t>
+          <t>فریدون شهر</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
@@ -2686,7 +2680,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>فریدن</t>
+          <t>فلاورجان</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
@@ -2716,7 +2710,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>فریدون شهر</t>
+          <t>کاشان</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
@@ -2746,7 +2740,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>فلاورجان</t>
+          <t>کوهپایه</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
@@ -2776,7 +2770,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>کوهپایه</t>
+          <t>گلپایگان</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
@@ -2806,7 +2800,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>گلپایگان</t>
+          <t>لنجان</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
@@ -2836,7 +2830,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>لنجان</t>
+          <t>مبارکه</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
@@ -3030,7 +3024,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
@@ -3040,119 +3034,119 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>مستندات عملکرد ۵ شاخص و حدود انتظار دوره ۲ ماهه به تفکیک شهرستان‌ها</t>
+          <t>ریز مستندات و اوزان شاخص‌های دوره ۲ ماهه به تفکیک شهرستان‌ها</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>نام ناحیه</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>نمره (۷۰-۱۰۰)</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>سطح</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>رتبه</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
-        <is>
-          <t>ماه‌های ارسالی</t>
-        </is>
-      </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>ماه‌ها</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>حوزه</t>
         </is>
       </c>
-      <c r="H3" s="11" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>انتظار حضوری</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>عملکرد حضوری</t>
         </is>
       </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="J3" s="9" t="inlineStr">
         <is>
           <t>تحقق حضوری</t>
         </is>
       </c>
-      <c r="K3" s="11" t="inlineStr">
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>انتظار مجازی</t>
         </is>
       </c>
-      <c r="L3" s="11" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t>عملکرد مجازی</t>
         </is>
       </c>
-      <c r="M3" s="11" t="inlineStr">
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>تحقق مجازی</t>
         </is>
       </c>
-      <c r="N3" s="11" t="inlineStr">
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>سهم آموزش (۴۰٪)</t>
+        </is>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>انتظار خلاقانه</t>
         </is>
       </c>
-      <c r="O3" s="11" t="inlineStr">
+      <c r="P3" s="9" t="inlineStr">
         <is>
           <t>عملکرد خلاقانه</t>
         </is>
       </c>
-      <c r="P3" s="11" t="inlineStr">
-        <is>
-          <t>تحقق خلاقانه</t>
-        </is>
-      </c>
-      <c r="Q3" s="11" t="inlineStr">
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>سهم خلاقانه (۵۰٪)</t>
+        </is>
+      </c>
+      <c r="R3" s="9" t="inlineStr">
         <is>
           <t>انتظار تولید</t>
         </is>
       </c>
-      <c r="R3" s="11" t="inlineStr">
+      <c r="S3" s="9" t="inlineStr">
         <is>
           <t>عملکرد تولید</t>
         </is>
       </c>
-      <c r="S3" s="11" t="inlineStr">
-        <is>
-          <t>تحقق تولید</t>
-        </is>
-      </c>
-      <c r="T3" s="11" t="inlineStr">
-        <is>
-          <t>تحقق کل</t>
+      <c r="T3" s="9" t="inlineStr">
+        <is>
+          <t>سهم تولید (۱۰٪)</t>
         </is>
       </c>
     </row>
@@ -3208,31 +3202,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N4" s="5" t="n">
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="n">
         <v>1240</v>
       </c>
-      <c r="O4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q4" s="5" t="n">
+      <c r="P4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="R4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S4" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T4" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -3288,31 +3282,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N5" s="5" t="n">
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="n">
         <v>620</v>
       </c>
-      <c r="O5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q5" s="5" t="n">
+      <c r="P5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="R5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S5" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -3326,19 +3320,21 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>عالی</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>1</v>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>2 از 2</t>
+          <t>0 از 2</t>
         </is>
       </c>
       <c r="G6" s="5" t="n">
@@ -3348,49 +3344,49 @@
         <v>1364</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>1400</v>
+        <v>0</v>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>102.6%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="K6" s="5" t="n">
         <v>9548</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>104.7%</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="n">
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="n">
         <v>2728</v>
       </c>
-      <c r="O6" s="5" t="n">
-        <v>2800</v>
-      </c>
-      <c r="P6" s="5" t="inlineStr">
-        <is>
-          <t>102.6%</t>
-        </is>
-      </c>
-      <c r="Q6" s="5" t="n">
+      <c r="P6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="n">
         <v>132</v>
       </c>
-      <c r="R6" s="5" t="n">
-        <v>140</v>
-      </c>
-      <c r="S6" s="5" t="inlineStr">
-        <is>
-          <t>106.1%</t>
-        </is>
+      <c r="S6" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T6" s="5" t="inlineStr">
         <is>
-          <t>103.2%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -3446,31 +3442,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N7" s="5" t="n">
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O7" s="5" t="n">
         <v>2728</v>
       </c>
-      <c r="O7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q7" s="5" t="n">
+      <c r="P7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="n">
         <v>132</v>
       </c>
-      <c r="R7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S7" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -3526,31 +3522,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N8" s="5" t="n">
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="n">
         <v>744</v>
       </c>
-      <c r="O8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q8" s="5" t="n">
+      <c r="P8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="R8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S8" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T8" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -3606,31 +3602,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N9" s="5" t="n">
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="n">
         <v>744</v>
       </c>
-      <c r="O9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q9" s="5" t="n">
+      <c r="P9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R9" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="R9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S9" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T9" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -3686,31 +3682,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N10" s="5" t="n">
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="n">
         <v>620</v>
       </c>
-      <c r="O10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q10" s="5" t="n">
+      <c r="P10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="R10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S10" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -3766,31 +3762,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N11" s="5" t="n">
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O11" s="5" t="n">
         <v>372</v>
       </c>
-      <c r="O11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q11" s="5" t="n">
+      <c r="P11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R11" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="R11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S11" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -3846,31 +3842,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N12" s="5" t="n">
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="n">
         <v>744</v>
       </c>
-      <c r="O12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q12" s="5" t="n">
+      <c r="P12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R12" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="R12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S12" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -3926,31 +3922,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N13" s="5" t="n">
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="n">
         <v>496</v>
       </c>
-      <c r="O13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q13" s="5" t="n">
+      <c r="P13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="R13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S13" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4006,31 +4002,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N14" s="5" t="n">
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="n">
         <v>620</v>
       </c>
-      <c r="O14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q14" s="5" t="n">
+      <c r="P14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R14" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="R14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S14" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4086,31 +4082,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N15" s="5" t="n">
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="n">
         <v>1116</v>
       </c>
-      <c r="O15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q15" s="5" t="n">
+      <c r="P15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="n">
         <v>54</v>
       </c>
-      <c r="R15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S15" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4166,31 +4162,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N16" s="5" t="n">
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="n">
         <v>372</v>
       </c>
-      <c r="O16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q16" s="5" t="n">
+      <c r="P16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="R16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S16" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4246,31 +4242,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N17" s="5" t="n">
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="n">
         <v>248</v>
       </c>
-      <c r="O17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q17" s="5" t="n">
+      <c r="P17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="R17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S17" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T17" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4326,31 +4322,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N18" s="5" t="n">
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="n">
         <v>496</v>
       </c>
-      <c r="O18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q18" s="5" t="n">
+      <c r="P18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="R18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S18" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4406,31 +4402,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N19" s="5" t="n">
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="n">
         <v>372</v>
       </c>
-      <c r="O19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q19" s="5" t="n">
+      <c r="P19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="R19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S19" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T19" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4486,31 +4482,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N20" s="5" t="n">
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="n">
         <v>868</v>
       </c>
-      <c r="O20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q20" s="5" t="n">
+      <c r="P20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="R20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S20" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T20" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4566,31 +4562,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N21" s="5" t="n">
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="n">
         <v>1116</v>
       </c>
-      <c r="O21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q21" s="5" t="n">
+      <c r="P21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="n">
         <v>54</v>
       </c>
-      <c r="R21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S21" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S21" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T21" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4646,31 +4642,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N22" s="5" t="n">
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="n">
         <v>992</v>
       </c>
-      <c r="O22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q22" s="5" t="n">
+      <c r="P22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="R22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S22" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T22" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4726,31 +4722,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N23" s="5" t="n">
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="n">
         <v>496</v>
       </c>
-      <c r="O23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q23" s="5" t="n">
+      <c r="P23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="R23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S23" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S23" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T23" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4806,31 +4802,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N24" s="5" t="n">
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="n">
         <v>372</v>
       </c>
-      <c r="O24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q24" s="5" t="n">
+      <c r="P24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="R24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S24" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S24" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T24" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4886,31 +4882,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N25" s="5" t="n">
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O25" s="5" t="n">
         <v>1364</v>
       </c>
-      <c r="O25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q25" s="5" t="n">
+      <c r="P25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="n">
         <v>66</v>
       </c>
-      <c r="R25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S25" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S25" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T25" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -4924,19 +4920,21 @@
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>2</v>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>1 از 2</t>
+          <t>0 از 2</t>
         </is>
       </c>
       <c r="G26" s="5" t="n">
@@ -4946,49 +4944,49 @@
         <v>930</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>53.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="K26" s="5" t="n">
         <v>6510</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>53.8%</t>
-        </is>
-      </c>
-      <c r="N26" s="5" t="n">
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="n">
         <v>1860</v>
       </c>
-      <c r="O26" s="5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="P26" s="5" t="inlineStr">
-        <is>
-          <t>53.8%</t>
-        </is>
-      </c>
-      <c r="Q26" s="5" t="n">
+      <c r="P26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="n">
         <v>90</v>
       </c>
-      <c r="R26" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="S26" s="5" t="inlineStr">
-        <is>
-          <t>55.6%</t>
-        </is>
+      <c r="S26" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T26" s="5" t="inlineStr">
         <is>
-          <t>53.4%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5044,31 +5042,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N27" s="5" t="n">
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O27" s="5" t="n">
         <v>496</v>
       </c>
-      <c r="O27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q27" s="5" t="n">
+      <c r="P27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R27" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="R27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S27" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S27" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T27" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5124,31 +5122,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N28" s="5" t="n">
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O28" s="5" t="n">
         <v>620</v>
       </c>
-      <c r="O28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q28" s="5" t="n">
+      <c r="P28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R28" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="R28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S28" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S28" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T28" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5204,31 +5202,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N29" s="5" t="n">
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O29" s="5" t="n">
         <v>1488</v>
       </c>
-      <c r="O29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q29" s="5" t="n">
+      <c r="P29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R29" s="5" t="n">
         <v>72</v>
       </c>
-      <c r="R29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S29" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S29" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T29" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5242,19 +5240,21 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>85.2</v>
+        <v>70</v>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="n">
-        <v>3</v>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>1 از 2</t>
+          <t>0 از 2</t>
         </is>
       </c>
       <c r="G30" s="5" t="n">
@@ -5264,49 +5264,49 @@
         <v>496</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>50.4%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="K30" s="5" t="n">
         <v>3472</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>50.4%</t>
-        </is>
-      </c>
-      <c r="N30" s="5" t="n">
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="N30" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O30" s="5" t="n">
         <v>992</v>
       </c>
-      <c r="O30" s="5" t="n">
-        <v>500</v>
-      </c>
-      <c r="P30" s="5" t="inlineStr">
-        <is>
-          <t>50.4%</t>
-        </is>
-      </c>
-      <c r="Q30" s="5" t="n">
+      <c r="P30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R30" s="5" t="n">
         <v>48</v>
       </c>
-      <c r="R30" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="S30" s="5" t="inlineStr">
-        <is>
-          <t>52.1%</t>
-        </is>
+      <c r="S30" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T30" s="5" t="inlineStr">
         <is>
-          <t>50.7%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5362,31 +5362,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N31" s="5" t="n">
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O31" s="5" t="n">
         <v>496</v>
       </c>
-      <c r="O31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q31" s="5" t="n">
+      <c r="P31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R31" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="R31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S31" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S31" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T31" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5442,31 +5442,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N32" s="5" t="n">
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O32" s="5" t="n">
         <v>1736</v>
       </c>
-      <c r="O32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P32" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q32" s="5" t="n">
+      <c r="P32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R32" s="5" t="n">
         <v>84</v>
       </c>
-      <c r="R32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S32" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S32" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T32" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5522,31 +5522,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N33" s="5" t="n">
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O33" s="5" t="n">
         <v>496</v>
       </c>
-      <c r="O33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q33" s="5" t="n">
+      <c r="P33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R33" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="R33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S33" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S33" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T33" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5602,31 +5602,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N34" s="5" t="n">
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O34" s="5" t="n">
         <v>248</v>
       </c>
-      <c r="O34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P34" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q34" s="5" t="n">
+      <c r="P34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R34" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="R34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S34" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S34" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T34" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5682,31 +5682,31 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="N35" s="5" t="n">
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="O35" s="5" t="n">
         <v>496</v>
       </c>
-      <c r="O35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="Q35" s="5" t="n">
+      <c r="P35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="5" t="inlineStr">
+        <is>
+          <t>0.00%</t>
+        </is>
+      </c>
+      <c r="R35" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="R35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S35" s="5" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
+      <c r="S35" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="T35" s="5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>

</xml_diff>